<commit_message>
Add design spec for int_medical_claim_lines_enriched
</commit_message>
<xml_diff>
--- a/docs/intermediate_model_curation.xlsx
+++ b/docs/intermediate_model_curation.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="28800" windowHeight="12240" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="int_member_plan_month_eligibili" sheetId="1" r:id="rId1"/>
+    <sheet name="int_medical_claim_lines_enriche" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="89">
   <si>
     <t>Model Definition</t>
   </si>
@@ -132,6 +133,169 @@
   </si>
   <si>
     <t>True when more than one segment contributes to the member-plan-month</t>
+  </si>
+  <si>
+    <t>MODEL:</t>
+  </si>
+  <si>
+    <t>int_medical_claim_lines_enriched</t>
+  </si>
+  <si>
+    <t>GRAIN:</t>
+  </si>
+  <si>
+    <t>claim_id + claim_line_number</t>
+  </si>
+  <si>
+    <t>SOURCE:</t>
+  </si>
+  <si>
+    <t>stg_medical_claim_lines + stg_eligibility_segments + stg_plans</t>
+  </si>
+  <si>
+    <t>PURPOSE:</t>
+  </si>
+  <si>
+    <t>Add member eligibility and plan context to medical claim lines</t>
+  </si>
+  <si>
+    <t>ATTRIBUTION RULE:</t>
+  </si>
+  <si>
+    <t>Claim lines are attributed to the eligibility segment containing service_from_date.</t>
+  </si>
+  <si>
+    <t>EXCEPTION RULE:</t>
+  </si>
+  <si>
+    <t>Claim lines without matching eligibility are retained and flagged for investigation.</t>
+  </si>
+  <si>
+    <t>ENRICHMENT:</t>
+  </si>
+  <si>
+    <t>Preserves claim-line fields and adds eligibility attribution and core plan context.</t>
+  </si>
+  <si>
+    <t>claim_id</t>
+  </si>
+  <si>
+    <t>unique_grain: Ensures each claim line appears only once after enrichment.
+row_count_matches_staging: Ensures enrichment does not add or remove claim lines.</t>
+  </si>
+  <si>
+    <t>claim_line_number</t>
+  </si>
+  <si>
+    <t>claim_type_code</t>
+  </si>
+  <si>
+    <t>claim_status_code</t>
+  </si>
+  <si>
+    <t>billing_provider_npi</t>
+  </si>
+  <si>
+    <t>rendering_provider_npi</t>
+  </si>
+  <si>
+    <t>billing_provider_type</t>
+  </si>
+  <si>
+    <t>bill_type_code</t>
+  </si>
+  <si>
+    <t>service_from_date</t>
+  </si>
+  <si>
+    <t>service_to_date</t>
+  </si>
+  <si>
+    <t>received_date</t>
+  </si>
+  <si>
+    <t>paid_date</t>
+  </si>
+  <si>
+    <t>place_of_service_code</t>
+  </si>
+  <si>
+    <t>revenue_code</t>
+  </si>
+  <si>
+    <t>procedure_code</t>
+  </si>
+  <si>
+    <t>procedure_modifier</t>
+  </si>
+  <si>
+    <t>units</t>
+  </si>
+  <si>
+    <t>diagnosis_code_1</t>
+  </si>
+  <si>
+    <t>diagnosis_code_2</t>
+  </si>
+  <si>
+    <t>diagnosis_code_3</t>
+  </si>
+  <si>
+    <t>billed_amount</t>
+  </si>
+  <si>
+    <t>allowed_amount</t>
+  </si>
+  <si>
+    <t>paid_amount</t>
+  </si>
+  <si>
+    <t>member_responsibility_amount</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>has_matching_eligibility</t>
+  </si>
+  <si>
+    <t>True when the claim line's service_from_date falls within an eligibility segment; otherwise false.</t>
+  </si>
+  <si>
+    <t>True when eligibility_segment_id is populated; otherwise false.</t>
+  </si>
+  <si>
+    <t>Ensures the eligibility-match flag agrees with whether an eligibility segment was matched.</t>
+  </si>
+  <si>
+    <t>eligibility_segment_id</t>
+  </si>
+  <si>
+    <t>Eligibility segment matched using service_from_date.</t>
+  </si>
+  <si>
+    <t>stg_eligibility_segments.eligibility_segment_id</t>
+  </si>
+  <si>
+    <t>Claim service_from_date must fall within the member's eligibility segment date range.</t>
+  </si>
+  <si>
+    <t>Ensures the matched eligibility segment belongs to the claim member and its date range includes the claim's service_from_date.</t>
+  </si>
+  <si>
+    <t>Plan associated with the eligibility segment matched using service_from_date.</t>
+  </si>
+  <si>
+    <t>plan_id must match the plan assigned to the matched eligibility segment.</t>
+  </si>
+  <si>
+    <t>state_code</t>
+  </si>
+  <si>
+    <t>product_code</t>
+  </si>
+  <si>
+    <t>aid_category_code</t>
   </si>
 </sst>
 </file>
@@ -144,7 +308,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,6 +320,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -631,151 +809,181 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1322,79 +1530,79 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="16.6666666666667" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.7777777777778" style="1" customWidth="1"/>
-    <col min="3" max="3" width="28.4444444444444" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44444444444444" style="2" customWidth="1"/>
-    <col min="5" max="5" width="8.33333333333333" style="2" customWidth="1"/>
-    <col min="6" max="6" width="23.8888888888889" style="1" customWidth="1"/>
-    <col min="7" max="7" width="37.5555555555556" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.7777777777778" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="1"/>
+    <col min="1" max="1" width="16.6666666666667" style="13" customWidth="1"/>
+    <col min="2" max="2" width="22.7777777777778" style="13" customWidth="1"/>
+    <col min="3" max="3" width="28.4444444444444" style="13" customWidth="1"/>
+    <col min="4" max="4" width="9.44444444444444" style="14" customWidth="1"/>
+    <col min="5" max="5" width="8.33333333333333" style="14" customWidth="1"/>
+    <col min="6" max="6" width="23.8888888888889" style="13" customWidth="1"/>
+    <col min="7" max="7" width="37.5555555555556" style="13" customWidth="1"/>
+    <col min="8" max="8" width="23.7777777777778" style="13" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:3">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="13" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:3">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="13" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:3">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="13" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:3">
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="5" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1405,10 +1613,10 @@
       <c r="C10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F10" s="4" t="s">
@@ -1424,10 +1632,10 @@
       <c r="C11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F11" s="4" t="s">
@@ -1443,10 +1651,10 @@
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="4"/>
@@ -1464,15 +1672,15 @@
       <c r="C13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6" t="s">
+      <c r="D13" s="16"/>
+      <c r="E13" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="4"/>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="17" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1483,8 +1691,8 @@
       <c r="C14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6" t="s">
+      <c r="D14" s="16"/>
+      <c r="E14" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="4"/>
@@ -1497,4 +1705,373 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="9.62962962962963" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.7777777777778" style="2" customWidth="1"/>
+    <col min="3" max="3" width="38.7592592592593" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9.44444444444444" style="3" customWidth="1"/>
+    <col min="5" max="5" width="8.33333333333333" style="3" customWidth="1"/>
+    <col min="6" max="6" width="25.5462962962963" style="4" customWidth="1"/>
+    <col min="7" max="7" width="40.6203703703704" style="4" customWidth="1"/>
+    <col min="8" max="8" width="45.1851851851852" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="2:3">
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3">
+      <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="B8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" s="1" customFormat="1" ht="32" customHeight="1" spans="2:8">
+      <c r="B12" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1" spans="2:8">
+      <c r="B13" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="8"/>
+    </row>
+    <row r="14" spans="2:6">
+      <c r="B14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="E14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3">
+      <c r="B15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="2:3">
+      <c r="B16" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="4"/>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="E21" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="4"/>
+    </row>
+    <row r="23" spans="2:3">
+      <c r="B23" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="4"/>
+    </row>
+    <row r="24" spans="2:3">
+      <c r="B24" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="4"/>
+    </row>
+    <row r="25" spans="2:3">
+      <c r="B25" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="4"/>
+    </row>
+    <row r="26" spans="2:3">
+      <c r="B26" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="4"/>
+    </row>
+    <row r="27" spans="2:3">
+      <c r="B27" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="4"/>
+    </row>
+    <row r="28" spans="2:3">
+      <c r="B28" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="4"/>
+    </row>
+    <row r="29" spans="2:3">
+      <c r="B29" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="4"/>
+    </row>
+    <row r="30" spans="2:3">
+      <c r="B30" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="4"/>
+    </row>
+    <row r="31" spans="2:3">
+      <c r="B31" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="4"/>
+    </row>
+    <row r="32" spans="2:3">
+      <c r="B32" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="2:3">
+      <c r="B33" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="4"/>
+    </row>
+    <row r="34" spans="2:3">
+      <c r="B34" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="2:3">
+      <c r="B35" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="2:3">
+      <c r="B36" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" spans="2:3">
+      <c r="B37" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" ht="43.2" spans="2:8">
+      <c r="B38" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" ht="28.8" spans="2:8">
+      <c r="B39" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" ht="28.8" spans="2:8">
+      <c r="B40" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H40" s="12"/>
+    </row>
+    <row r="41" spans="2:8">
+      <c r="B41" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="H41" s="12"/>
+    </row>
+    <row r="42" spans="2:8">
+      <c r="B42" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C42" s="4"/>
+      <c r="H42" s="12"/>
+    </row>
+    <row r="43" spans="2:8">
+      <c r="B43" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C43" s="4"/>
+      <c r="H43" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="H39:H43"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add int_medical_claim_lines_enriched with tests
</commit_message>
<xml_diff>
--- a/docs/intermediate_model_curation.xlsx
+++ b/docs/intermediate_model_curation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12240" activeTab="1"/>
+    <workbookView windowWidth="20184" windowHeight="12240" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="int_member_plan_month_eligibili" sheetId="1" r:id="rId1"/>
@@ -265,7 +265,21 @@
     <t>True when eligibility_segment_id is populated; otherwise false.</t>
   </si>
   <si>
-    <t>Ensures the eligibility-match flag agrees with whether an eligibility segment was matched.</t>
+    <r>
+      <t xml:space="preserve">Test not needed for otherwise tautological test: </t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Ensures the eligibility-match flag agrees with whether an eligibility segment was matched. 
+</t>
+    </r>
   </si>
   <si>
     <t>eligibility_segment_id</t>
@@ -280,7 +294,21 @@
     <t>Claim service_from_date must fall within the member's eligibility segment date range.</t>
   </si>
   <si>
-    <t>Ensures the matched eligibility segment belongs to the claim member and its date range includes the claim's service_from_date.</t>
+    <r>
+      <t xml:space="preserve">Test not needed for otherwise tautological test: 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <strike/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ensures the matched eligibility segment belongs to the claim member and its date range includes the claim's service_from_date.</t>
+    </r>
   </si>
   <si>
     <t>Plan associated with the eligibility segment matched using service_from_date.</t>
@@ -308,7 +336,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -482,13 +510,27 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFED5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -815,7 +857,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -839,16 +881,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -857,89 +899,89 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -967,16 +1009,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -985,13 +1039,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1261,6 +1315,12 @@
       <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="00FFFE93"/>
+      <color rgb="00FFFED5"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1530,56 +1590,56 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="16.6666666666667" style="13" customWidth="1"/>
-    <col min="2" max="2" width="22.7777777777778" style="13" customWidth="1"/>
-    <col min="3" max="3" width="28.4444444444444" style="13" customWidth="1"/>
-    <col min="4" max="4" width="9.44444444444444" style="14" customWidth="1"/>
-    <col min="5" max="5" width="8.33333333333333" style="14" customWidth="1"/>
-    <col min="6" max="6" width="23.8888888888889" style="13" customWidth="1"/>
-    <col min="7" max="7" width="37.5555555555556" style="13" customWidth="1"/>
-    <col min="8" max="8" width="23.7777777777778" style="13" customWidth="1"/>
-    <col min="9" max="16384" width="8.88888888888889" style="13"/>
+    <col min="1" max="1" width="16.6666666666667" style="17" customWidth="1"/>
+    <col min="2" max="2" width="22.7777777777778" style="17" customWidth="1"/>
+    <col min="3" max="3" width="28.4444444444444" style="17" customWidth="1"/>
+    <col min="4" max="4" width="9.44444444444444" style="18" customWidth="1"/>
+    <col min="5" max="5" width="8.33333333333333" style="18" customWidth="1"/>
+    <col min="6" max="6" width="23.8888888888889" style="17" customWidth="1"/>
+    <col min="7" max="7" width="37.5555555555556" style="17" customWidth="1"/>
+    <col min="8" max="8" width="23.7777777777778" style="17" customWidth="1"/>
+    <col min="9" max="16384" width="8.88888888888889" style="17"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="2:3">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="17" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="2:3">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="17" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:3">
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="17" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:3">
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="17" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="17" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1613,10 +1673,10 @@
       <c r="C10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F10" s="4" t="s">
@@ -1632,10 +1692,10 @@
       <c r="C11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F11" s="4" t="s">
@@ -1651,10 +1711,10 @@
       <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="4"/>
@@ -1672,15 +1732,15 @@
       <c r="C13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16" t="s">
+      <c r="D13" s="20"/>
+      <c r="E13" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="4"/>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="H13" s="21" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1691,8 +1751,8 @@
       <c r="C14" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16" t="s">
+      <c r="D14" s="20"/>
+      <c r="E14" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F14" s="4"/>
@@ -1718,8 +1778,8 @@
     <col min="3" max="3" width="38.7592592592593" style="2" customWidth="1"/>
     <col min="4" max="4" width="9.44444444444444" style="3" customWidth="1"/>
     <col min="5" max="5" width="8.33333333333333" style="3" customWidth="1"/>
-    <col min="6" max="6" width="25.5462962962963" style="4" customWidth="1"/>
-    <col min="7" max="7" width="40.6203703703704" style="4" customWidth="1"/>
+    <col min="6" max="6" width="25.5462962962963" style="4" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="40.6203703703704" style="4" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="45.1851851851852" style="4" customWidth="1"/>
     <col min="9" max="16384" width="8.88888888888889" style="2"/>
   </cols>
@@ -1821,30 +1881,30 @@
       <c r="D12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="10" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="11" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="2:8">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="12" t="s">
         <v>51</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="13" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="8"/>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" spans="2:6">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="12" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="4"/>
@@ -1856,43 +1916,43 @@
       </c>
     </row>
     <row r="15" spans="2:3">
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="12" t="s">
         <v>52</v>
       </c>
       <c r="C15" s="4"/>
     </row>
     <row r="16" spans="2:3">
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="12" t="s">
         <v>53</v>
       </c>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="2:3">
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="12" t="s">
         <v>54</v>
       </c>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="2:3">
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="12" t="s">
         <v>55</v>
       </c>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="2:3">
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="12" t="s">
         <v>56</v>
       </c>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="2:3">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="12" t="s">
         <v>57</v>
       </c>
       <c r="C20" s="4"/>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="12" t="s">
         <v>58</v>
       </c>
       <c r="C21" s="4"/>
@@ -1901,103 +1961,103 @@
       </c>
     </row>
     <row r="22" spans="2:3">
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="12" t="s">
         <v>59</v>
       </c>
       <c r="C22" s="4"/>
     </row>
     <row r="23" spans="2:3">
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="12" t="s">
         <v>60</v>
       </c>
       <c r="C23" s="4"/>
     </row>
     <row r="24" spans="2:3">
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="12" t="s">
         <v>61</v>
       </c>
       <c r="C24" s="4"/>
     </row>
     <row r="25" spans="2:3">
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="12" t="s">
         <v>62</v>
       </c>
       <c r="C25" s="4"/>
     </row>
     <row r="26" spans="2:3">
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="12" t="s">
         <v>63</v>
       </c>
       <c r="C26" s="4"/>
     </row>
     <row r="27" spans="2:3">
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="12" t="s">
         <v>64</v>
       </c>
       <c r="C27" s="4"/>
     </row>
     <row r="28" spans="2:3">
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="12" t="s">
         <v>65</v>
       </c>
       <c r="C28" s="4"/>
     </row>
     <row r="29" spans="2:3">
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="12" t="s">
         <v>66</v>
       </c>
       <c r="C29" s="4"/>
     </row>
     <row r="30" spans="2:3">
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="12" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="4"/>
     </row>
     <row r="31" spans="2:3">
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="12" t="s">
         <v>68</v>
       </c>
       <c r="C31" s="4"/>
     </row>
     <row r="32" spans="2:3">
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="12" t="s">
         <v>69</v>
       </c>
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="2:3">
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="12" t="s">
         <v>70</v>
       </c>
       <c r="C33" s="4"/>
     </row>
     <row r="34" spans="2:3">
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="12" t="s">
         <v>71</v>
       </c>
       <c r="C34" s="4"/>
     </row>
     <row r="35" spans="2:3">
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="12" t="s">
         <v>72</v>
       </c>
       <c r="C35" s="4"/>
     </row>
     <row r="36" spans="2:3">
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="12" t="s">
         <v>73</v>
       </c>
       <c r="C36" s="4"/>
     </row>
     <row r="37" spans="2:3">
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="12" t="s">
         <v>74</v>
       </c>
       <c r="C37" s="4"/>
     </row>
-    <row r="38" ht="43.2" spans="2:8">
-      <c r="B38" s="11" t="s">
+    <row r="38" ht="57.6" spans="2:8">
+      <c r="B38" s="14" t="s">
         <v>75</v>
       </c>
       <c r="C38" s="4" t="s">
@@ -2009,12 +2069,12 @@
       <c r="G38" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H38" s="4" t="s">
+      <c r="H38" s="15" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="39" ht="28.8" spans="2:8">
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="14" t="s">
         <v>79</v>
       </c>
       <c r="C39" s="4" t="s">
@@ -2026,12 +2086,12 @@
       <c r="G39" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H39" s="12" t="s">
+      <c r="H39" s="11" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="40" ht="28.8" spans="2:8">
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C40" s="4" t="s">
@@ -2043,28 +2103,28 @@
       <c r="G40" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="H40" s="12"/>
+      <c r="H40" s="16"/>
     </row>
     <row r="41" spans="2:8">
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C41" s="4"/>
-      <c r="H41" s="12"/>
+      <c r="H41" s="16"/>
     </row>
     <row r="42" spans="2:8">
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="14" t="s">
         <v>87</v>
       </c>
       <c r="C42" s="4"/>
-      <c r="H42" s="12"/>
+      <c r="H42" s="16"/>
     </row>
     <row r="43" spans="2:8">
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="14" t="s">
         <v>88</v>
       </c>
       <c r="C43" s="4"/>
-      <c r="H43" s="12"/>
+      <c r="H43" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add design spec for fct_member_plan_month
Mark int_member_plan_month_eligibility as replaced in the intermediate spec.
</commit_message>
<xml_diff>
--- a/docs/intermediate_model_curation.xlsx
+++ b/docs/intermediate_model_curation.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20184" windowHeight="12240" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12240"/>
   </bookViews>
   <sheets>
     <sheet name="int_member_plan_month_eligibili" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
+  <si>
+    <t>Note on 10/7/2026: int_member_plan_month_eligibility is replaced by fct_member_plan_month</t>
+  </si>
   <si>
     <t>Model Definition</t>
   </si>
@@ -266,6 +269,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Test not needed for otherwise tautological test: </t>
     </r>
     <r>
@@ -295,6 +305,13 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Test not needed for otherwise tautological test: 
 </t>
     </r>
@@ -336,7 +353,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,6 +379,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -851,137 +875,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1038,6 +1062,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1587,7 +1614,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="16.6666666666667" style="17" customWidth="1"/>
@@ -1602,164 +1629,169 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:3">
-      <c r="B2" s="17" t="s">
+    <row r="3" spans="1:1">
+      <c r="A3" s="17" t="s">
         <v>1</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="2:3">
-      <c r="B3" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="17" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3">
+      <c r="B6" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="17" t="s">
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" s="17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="17" t="s">
+      <c r="C7" s="17" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:8">
-      <c r="B9" s="5" t="s">
+    <row r="10" spans="1:1">
+      <c r="A10" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="5" t="s">
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="2:8">
-      <c r="B10" s="4" t="s">
+      <c r="H11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="2:8">
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
     </row>
     <row r="12" spans="2:8">
       <c r="B12" s="4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>27</v>
-      </c>
+      <c r="D12" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="13" spans="2:8">
       <c r="B13" s="4" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="H13" s="21" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" ht="28.8" spans="2:8">
+        <v>23</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="2:8">
       <c r="B14" s="4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>20</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="G15" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" ht="28.8" spans="2:8">
+      <c r="B16" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H14" s="4"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1786,342 +1818,342 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="2:3">
       <c r="B2" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="B11" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="1" ht="32" customHeight="1" spans="2:8">
       <c r="B12" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="2:8">
       <c r="B13" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H13" s="11"/>
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C14" s="4"/>
       <c r="E14" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="2:3">
       <c r="B15" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C15" s="4"/>
     </row>
     <row r="16" spans="2:3">
       <c r="B16" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="2:3">
       <c r="B17" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="2:3">
       <c r="B18" s="12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="2:3">
       <c r="B19" s="12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="2:3">
       <c r="B20" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" s="4"/>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C21" s="4"/>
       <c r="E21" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="2:3">
       <c r="B22" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" s="4"/>
     </row>
     <row r="23" spans="2:3">
       <c r="B23" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C23" s="4"/>
     </row>
     <row r="24" spans="2:3">
       <c r="B24" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="4"/>
     </row>
     <row r="25" spans="2:3">
       <c r="B25" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="4"/>
     </row>
     <row r="26" spans="2:3">
       <c r="B26" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C26" s="4"/>
     </row>
     <row r="27" spans="2:3">
       <c r="B27" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C27" s="4"/>
     </row>
     <row r="28" spans="2:3">
       <c r="B28" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C28" s="4"/>
     </row>
     <row r="29" spans="2:3">
       <c r="B29" s="12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C29" s="4"/>
     </row>
     <row r="30" spans="2:3">
       <c r="B30" s="12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C30" s="4"/>
     </row>
     <row r="31" spans="2:3">
       <c r="B31" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C31" s="4"/>
     </row>
     <row r="32" spans="2:3">
       <c r="B32" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C32" s="4"/>
     </row>
     <row r="33" spans="2:3">
       <c r="B33" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C33" s="4"/>
     </row>
     <row r="34" spans="2:3">
       <c r="B34" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C34" s="4"/>
     </row>
     <row r="35" spans="2:3">
       <c r="B35" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C35" s="4"/>
     </row>
     <row r="36" spans="2:3">
       <c r="B36" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C36" s="4"/>
     </row>
     <row r="37" spans="2:3">
       <c r="B37" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C37" s="4"/>
     </row>
     <row r="38" ht="57.6" spans="2:8">
       <c r="B38" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H38" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" ht="28.8" spans="2:8">
       <c r="B39" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H39" s="11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" ht="28.8" spans="2:8">
       <c r="B40" s="14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H40" s="16"/>
     </row>
     <row r="41" spans="2:8">
       <c r="B41" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C41" s="4"/>
       <c r="H41" s="16"/>
     </row>
     <row r="42" spans="2:8">
       <c r="B42" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C42" s="4"/>
       <c r="H42" s="16"/>
     </row>
     <row r="43" spans="2:8">
       <c r="B43" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C43" s="4"/>
       <c r="H43" s="16"/>

</xml_diff>